<commit_message>
pruebas iniciales filtro Kalman
</commit_message>
<xml_diff>
--- a/Test_ESP_Now/Test_Analisis_de_RSSI/Analisis desviacion.xlsx
+++ b/Test_ESP_Now/Test_Analisis_de_RSSI/Analisis desviacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://itba2-my.sharepoint.com/personal/tgreco_itba_edu_ar/Documents/ITBA/Tesis/ProyectoFinal/Test_ESP_Now/Test_Analisis_de_RSSI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="11_F25DC773A252ABDACC10483599DA60A25ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6BB9327-CA4A-4E74-A893-22E252AF95C7}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="11_F25DC773A252ABDACC10483599DA60A25ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1FD4C2EC-B6CC-4C36-A50F-72D2BF26BBED}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3081,6 +3081,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" connectionId="2" xr16:uid="{B40D9AFC-F734-4BCE-999F-3C19EA4CA6AB}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="3">
@@ -5923,7 +5927,7 @@
         <v>-52</v>
       </c>
       <c r="D210">
-        <f t="shared" ref="D210:D229" si="9">AVERAGE(B210:B219)</f>
+        <f t="shared" ref="D210:D227" si="9">AVERAGE(B210:B219)</f>
         <v>-52.9</v>
       </c>
     </row>
@@ -11539,7 +11543,7 @@
         <v>-51</v>
       </c>
       <c r="D678">
-        <f t="shared" ref="D678:D701" si="17">AVERAGE(B678:B687)</f>
+        <f t="shared" ref="D678:D691" si="17">AVERAGE(B678:B687)</f>
         <v>-52.4</v>
       </c>
     </row>

</xml_diff>